<commit_message>
Removes extra rows from plcy-schd/V CSVs
</commit_message>
<xml_diff>
--- a/InputData/plcy-schd/V/Vintage.xlsx
+++ b/InputData/plcy-schd/V/Vintage.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\plcy-schd\V\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD24F716-DF92-4A8B-9F59-A270CC7C5B76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A7A55AB-7E12-459F-B36D-DB5D5E1386B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="27270" windowHeight="16395" activeTab="5" xr2:uid="{70679913-52CE-4866-92D3-04053F7F27F8}"/>
+    <workbookView xWindow="29580" yWindow="780" windowWidth="21600" windowHeight="11175" activeTab="1" xr2:uid="{70679913-52CE-4866-92D3-04053F7F27F8}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -516,7 +516,7 @@
   <sheetPr>
     <tabColor theme="3" tint="9.9978637043366805E-2"/>
   </sheetPr>
-  <dimension ref="A1:A174"/>
+  <dimension ref="A1:A152"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1428,138 +1428,6 @@
       <c r="A152" t="str">
         <f>IF(About!$A$9+ROW(A150)&gt;About!$A$10,"","Vintage"&amp;About!$A$9+ROW(A150))</f>
         <v>Vintage2100</v>
-      </c>
-    </row>
-    <row r="153" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A153" t="str">
-        <f>IF(About!$A$9+ROW(A151)&gt;About!$A$10,"","Vintage"&amp;About!$A$9+ROW(A151))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="154" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A154" t="str">
-        <f>IF(About!$A$9+ROW(A152)&gt;About!$A$10,"","Vintage"&amp;About!$A$9+ROW(A152))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="155" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A155" t="str">
-        <f>IF(About!$A$9+ROW(A153)&gt;About!$A$10,"","Vintage"&amp;About!$A$9+ROW(A153))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="156" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A156" t="str">
-        <f>IF(About!$A$9+ROW(A154)&gt;About!$A$10,"","Vintage"&amp;About!$A$9+ROW(A154))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="157" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A157" t="str">
-        <f>IF(About!$A$9+ROW(A155)&gt;About!$A$10,"","Vintage"&amp;About!$A$9+ROW(A155))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="158" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A158" t="str">
-        <f>IF(About!$A$9+ROW(A156)&gt;About!$A$10,"","Vintage"&amp;About!$A$9+ROW(A156))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="159" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A159" t="str">
-        <f>IF(About!$A$9+ROW(A157)&gt;About!$A$10,"","Vintage"&amp;About!$A$9+ROW(A157))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="160" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A160" t="str">
-        <f>IF(About!$A$9+ROW(A158)&gt;About!$A$10,"","Vintage"&amp;About!$A$9+ROW(A158))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="161" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A161" t="str">
-        <f>IF(About!$A$9+ROW(A159)&gt;About!$A$10,"","Vintage"&amp;About!$A$9+ROW(A159))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="162" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A162" t="str">
-        <f>IF(About!$A$9+ROW(A160)&gt;About!$A$10,"","Vintage"&amp;About!$A$9+ROW(A160))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="163" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A163" t="str">
-        <f>IF(About!$A$9+ROW(A161)&gt;About!$A$10,"","Vintage"&amp;About!$A$9+ROW(A161))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="164" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A164" t="str">
-        <f>IF(About!$A$9+ROW(A162)&gt;About!$A$10,"","Vintage"&amp;About!$A$9+ROW(A162))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="165" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A165" t="str">
-        <f>IF(About!$A$9+ROW(A163)&gt;About!$A$10,"","Vintage"&amp;About!$A$9+ROW(A163))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="166" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A166" t="str">
-        <f>IF(About!$A$9+ROW(A164)&gt;About!$A$10,"","Vintage"&amp;About!$A$9+ROW(A164))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="167" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A167" t="str">
-        <f>IF(About!$A$9+ROW(A165)&gt;About!$A$10,"","Vintage"&amp;About!$A$9+ROW(A165))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="168" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A168" t="str">
-        <f>IF(About!$A$9+ROW(A166)&gt;About!$A$10,"","Vintage"&amp;About!$A$9+ROW(A166))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="169" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A169" t="str">
-        <f>IF(About!$A$9+ROW(A167)&gt;About!$A$10,"","Vintage"&amp;About!$A$9+ROW(A167))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="170" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A170" t="str">
-        <f>IF(About!$A$9+ROW(A168)&gt;About!$A$10,"","Vintage"&amp;About!$A$9+ROW(A168))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="171" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A171" t="str">
-        <f>IF(About!$A$9+ROW(A169)&gt;About!$A$10,"","Vintage"&amp;About!$A$9+ROW(A169))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="172" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A172" t="str">
-        <f>IF(About!$A$9+ROW(A170)&gt;About!$A$10,"","Vintage"&amp;About!$A$9+ROW(A170))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="173" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A173" t="str">
-        <f>IF(About!$A$9+ROW(A171)&gt;About!$A$10,"","Vintage"&amp;About!$A$9+ROW(A171))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="174" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A174" t="str">
-        <f>IF(About!$A$9+ROW(A172)&gt;About!$A$10,"","Vintage"&amp;About!$A$9+ROW(A172))</f>
-        <v/>
       </c>
     </row>
   </sheetData>
@@ -1596,7 +1464,7 @@
   <sheetPr>
     <tabColor theme="3" tint="9.9978637043366805E-2"/>
   </sheetPr>
-  <dimension ref="A1:A173"/>
+  <dimension ref="A1:A151"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -2502,138 +2370,6 @@
       <c r="A151" t="str">
         <f>V!A152</f>
         <v>Vintage2100</v>
-      </c>
-    </row>
-    <row r="152" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A152" t="str">
-        <f>V!A153</f>
-        <v/>
-      </c>
-    </row>
-    <row r="153" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A153" t="str">
-        <f>V!A154</f>
-        <v/>
-      </c>
-    </row>
-    <row r="154" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A154" t="str">
-        <f>V!A155</f>
-        <v/>
-      </c>
-    </row>
-    <row r="155" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A155" t="str">
-        <f>V!A156</f>
-        <v/>
-      </c>
-    </row>
-    <row r="156" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A156" t="str">
-        <f>V!A157</f>
-        <v/>
-      </c>
-    </row>
-    <row r="157" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A157" t="str">
-        <f>V!A158</f>
-        <v/>
-      </c>
-    </row>
-    <row r="158" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A158" t="str">
-        <f>V!A159</f>
-        <v/>
-      </c>
-    </row>
-    <row r="159" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A159" t="str">
-        <f>V!A160</f>
-        <v/>
-      </c>
-    </row>
-    <row r="160" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A160" t="str">
-        <f>V!A161</f>
-        <v/>
-      </c>
-    </row>
-    <row r="161" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A161" t="str">
-        <f>V!A162</f>
-        <v/>
-      </c>
-    </row>
-    <row r="162" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A162" t="str">
-        <f>V!A163</f>
-        <v/>
-      </c>
-    </row>
-    <row r="163" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A163" t="str">
-        <f>V!A164</f>
-        <v/>
-      </c>
-    </row>
-    <row r="164" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A164" t="str">
-        <f>V!A165</f>
-        <v/>
-      </c>
-    </row>
-    <row r="165" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A165" t="str">
-        <f>V!A166</f>
-        <v/>
-      </c>
-    </row>
-    <row r="166" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A166" t="str">
-        <f>V!A167</f>
-        <v/>
-      </c>
-    </row>
-    <row r="167" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A167" t="str">
-        <f>V!A168</f>
-        <v/>
-      </c>
-    </row>
-    <row r="168" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A168" t="str">
-        <f>V!A169</f>
-        <v/>
-      </c>
-    </row>
-    <row r="169" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A169" t="str">
-        <f>V!A170</f>
-        <v/>
-      </c>
-    </row>
-    <row r="170" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A170" t="str">
-        <f>V!A171</f>
-        <v/>
-      </c>
-    </row>
-    <row r="171" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A171" t="str">
-        <f>V!A172</f>
-        <v/>
-      </c>
-    </row>
-    <row r="172" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A172" t="str">
-        <f>V!A173</f>
-        <v/>
-      </c>
-    </row>
-    <row r="173" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A173" t="str">
-        <f>V!A174</f>
-        <v/>
       </c>
     </row>
   </sheetData>
@@ -2646,7 +2382,7 @@
   <sheetPr>
     <tabColor theme="3" tint="9.9978637043366805E-2"/>
   </sheetPr>
-  <dimension ref="A1:A252"/>
+  <dimension ref="A1:A151"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -3552,612 +3288,6 @@
       <c r="A151" t="str">
         <f>IF(V!A152="","",V!A151)</f>
         <v>Vintage2099</v>
-      </c>
-    </row>
-    <row r="152" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A152" t="str">
-        <f>IF(V!A153="","",V!A152)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="153" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A153" t="str">
-        <f>IF(V!A154="","",V!A153)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="154" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A154" t="str">
-        <f>IF(V!A155="","",V!A154)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="155" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A155" t="str">
-        <f>IF(V!A156="","",V!A155)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="156" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A156" t="str">
-        <f>IF(V!A157="","",V!A156)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="157" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A157" t="str">
-        <f>IF(V!A158="","",V!A157)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="158" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A158" t="str">
-        <f>IF(V!A159="","",V!A158)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="159" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A159" t="str">
-        <f>IF(V!A160="","",V!A159)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="160" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A160" t="str">
-        <f>IF(V!A161="","",V!A160)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="161" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A161" t="str">
-        <f>IF(V!A162="","",V!A161)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="162" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A162" t="str">
-        <f>IF(V!A163="","",V!A162)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="163" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A163" t="str">
-        <f>IF(V!A164="","",V!A163)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="164" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A164" t="str">
-        <f>IF(V!A165="","",V!A164)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="165" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A165" t="str">
-        <f>IF(V!A166="","",V!A165)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="166" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A166" t="str">
-        <f>IF(V!A167="","",V!A166)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="167" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A167" t="str">
-        <f>IF(V!A168="","",V!A167)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="168" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A168" t="str">
-        <f>IF(V!A169="","",V!A168)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="169" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A169" t="str">
-        <f>IF(V!A170="","",V!A169)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="170" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A170" t="str">
-        <f>IF(V!A171="","",V!A170)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="171" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A171" t="str">
-        <f>IF(V!A172="","",V!A171)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="172" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A172" t="str">
-        <f>IF(V!A173="","",V!A172)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="173" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A173" t="str">
-        <f>IF(V!A174="","",V!A173)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="174" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A174" t="str">
-        <f>IF(V!A175="","",V!A174)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="175" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A175" t="str">
-        <f>IF(V!A176="","",V!A175)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="176" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A176" t="str">
-        <f>IF(V!A177="","",V!A176)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="177" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A177" t="str">
-        <f>IF(V!A178="","",V!A177)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="178" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A178" t="str">
-        <f>IF(V!A179="","",V!A178)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="179" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A179" t="str">
-        <f>IF(V!A180="","",V!A179)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="180" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A180" t="str">
-        <f>IF(V!A181="","",V!A180)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="181" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A181" t="str">
-        <f>IF(V!A182="","",V!A181)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="182" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A182" t="str">
-        <f>IF(V!A183="","",V!A182)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="183" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A183" t="str">
-        <f>IF(V!A184="","",V!A183)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="184" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A184" t="str">
-        <f>IF(V!A185="","",V!A184)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="185" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A185" t="str">
-        <f>IF(V!A186="","",V!A185)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="186" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A186" t="str">
-        <f>IF(V!A187="","",V!A186)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="187" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A187" t="str">
-        <f>IF(V!A188="","",V!A187)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="188" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A188" t="str">
-        <f>IF(V!A189="","",V!A188)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="189" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A189" t="str">
-        <f>IF(V!A190="","",V!A189)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="190" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A190" t="str">
-        <f>IF(V!A191="","",V!A190)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="191" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A191" t="str">
-        <f>IF(V!A192="","",V!A191)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="192" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A192" t="str">
-        <f>IF(V!A193="","",V!A192)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="193" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A193" t="str">
-        <f>IF(V!A194="","",V!A193)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="194" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A194" t="str">
-        <f>IF(V!A195="","",V!A194)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="195" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A195" t="str">
-        <f>IF(V!A196="","",V!A195)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="196" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A196" t="str">
-        <f>IF(V!A197="","",V!A196)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="197" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A197" t="str">
-        <f>IF(V!A198="","",V!A197)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="198" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A198" t="str">
-        <f>IF(V!A199="","",V!A198)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="199" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A199" t="str">
-        <f>IF(V!A200="","",V!A199)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="200" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A200" t="str">
-        <f>IF(V!A201="","",V!A200)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="201" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A201" t="str">
-        <f>IF(V!A202="","",V!A201)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="202" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A202" t="str">
-        <f>IF(V!A203="","",V!A202)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="203" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A203" t="str">
-        <f>IF(V!A204="","",V!A203)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="204" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A204" t="str">
-        <f>IF(V!A205="","",V!A204)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="205" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A205" t="str">
-        <f>IF(V!A206="","",V!A205)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="206" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A206" t="str">
-        <f>IF(V!A207="","",V!A206)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="207" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A207" t="str">
-        <f>IF(V!A208="","",V!A207)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="208" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A208" t="str">
-        <f>IF(V!A209="","",V!A208)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="209" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A209" t="str">
-        <f>IF(V!A210="","",V!A209)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="210" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A210" t="str">
-        <f>IF(V!A211="","",V!A210)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="211" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A211" t="str">
-        <f>IF(V!A212="","",V!A211)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="212" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A212" t="str">
-        <f>IF(V!A213="","",V!A212)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="213" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A213" t="str">
-        <f>IF(V!A214="","",V!A213)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="214" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A214" t="str">
-        <f>IF(V!A215="","",V!A214)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="215" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A215" t="str">
-        <f>IF(V!A216="","",V!A215)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="216" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A216" t="str">
-        <f>IF(V!A217="","",V!A216)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="217" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A217" t="str">
-        <f>IF(V!A218="","",V!A217)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="218" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A218" t="str">
-        <f>IF(V!A219="","",V!A218)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="219" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A219" t="str">
-        <f>IF(V!A220="","",V!A219)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="220" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A220" t="str">
-        <f>IF(V!A221="","",V!A220)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="221" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A221" t="str">
-        <f>IF(V!A222="","",V!A221)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="222" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A222" t="str">
-        <f>IF(V!A223="","",V!A222)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="223" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A223" t="str">
-        <f>IF(V!A224="","",V!A223)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="224" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A224" t="str">
-        <f>IF(V!A225="","",V!A224)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="225" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A225" t="str">
-        <f>IF(V!A226="","",V!A225)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="226" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A226" t="str">
-        <f>IF(V!A227="","",V!A226)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="227" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A227" t="str">
-        <f>IF(V!A228="","",V!A227)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="228" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A228" t="str">
-        <f>IF(V!A229="","",V!A228)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="229" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A229" t="str">
-        <f>IF(V!A230="","",V!A229)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="230" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A230" t="str">
-        <f>IF(V!A231="","",V!A230)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="231" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A231" t="str">
-        <f>IF(V!A232="","",V!A231)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="232" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A232" t="str">
-        <f>IF(V!A233="","",V!A232)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="233" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A233" t="str">
-        <f>IF(V!A234="","",V!A233)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="234" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A234" t="str">
-        <f>IF(V!A235="","",V!A234)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="235" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A235" t="str">
-        <f>IF(V!A236="","",V!A235)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="236" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A236" t="str">
-        <f>IF(V!A237="","",V!A236)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="237" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A237" t="str">
-        <f>IF(V!A238="","",V!A237)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="238" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A238" t="str">
-        <f>IF(V!A239="","",V!A238)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="239" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A239" t="str">
-        <f>IF(V!A240="","",V!A239)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="240" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A240" t="str">
-        <f>IF(V!A241="","",V!A240)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="241" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A241" t="str">
-        <f>IF(V!A242="","",V!A241)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="242" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A242" t="str">
-        <f>IF(V!A243="","",V!A242)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="243" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A243" t="str">
-        <f>IF(V!A244="","",V!A243)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="244" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A244" t="str">
-        <f>IF(V!A245="","",V!A244)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="245" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A245" t="str">
-        <f>IF(V!A246="","",V!A245)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="246" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A246" t="str">
-        <f>IF(V!A247="","",V!A246)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="247" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A247" t="str">
-        <f>IF(V!A248="","",V!A247)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="248" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A248" t="str">
-        <f>IF(V!A249="","",V!A248)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="249" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A249" t="str">
-        <f>IF(V!A250="","",V!A249)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="250" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A250" t="str">
-        <f>IF(V!A251="","",V!A250)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="251" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A251" t="str">
-        <f>IF(V!A252="","",V!A251)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="252" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A252" t="str">
-        <f>IF(V!A253="","",V!A252)</f>
-        <v/>
       </c>
     </row>
   </sheetData>
@@ -4170,7 +3300,7 @@
   <sheetPr>
     <tabColor theme="3" tint="9.9978637043366805E-2"/>
   </sheetPr>
-  <dimension ref="A1:A94"/>
+  <dimension ref="A1:A72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -4603,138 +3733,6 @@
         <v>Vintage2020</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A73" t="str">
-        <f>V!A153</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A74" t="str">
-        <f>V!A154</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A75" t="str">
-        <f>V!A155</f>
-        <v/>
-      </c>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A76" t="str">
-        <f>V!A156</f>
-        <v/>
-      </c>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A77" t="str">
-        <f>V!A157</f>
-        <v/>
-      </c>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A78" t="str">
-        <f>V!A158</f>
-        <v/>
-      </c>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A79" t="str">
-        <f>V!A159</f>
-        <v/>
-      </c>
-    </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A80" t="str">
-        <f>V!A160</f>
-        <v/>
-      </c>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A81" t="str">
-        <f>V!A161</f>
-        <v/>
-      </c>
-    </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A82" t="str">
-        <f>V!A162</f>
-        <v/>
-      </c>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A83" t="str">
-        <f>V!A163</f>
-        <v/>
-      </c>
-    </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A84" t="str">
-        <f>V!A164</f>
-        <v/>
-      </c>
-    </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A85" t="str">
-        <f>V!A165</f>
-        <v/>
-      </c>
-    </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A86" t="str">
-        <f>V!A166</f>
-        <v/>
-      </c>
-    </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A87" t="str">
-        <f>V!A167</f>
-        <v/>
-      </c>
-    </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A88" t="str">
-        <f>V!A168</f>
-        <v/>
-      </c>
-    </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A89" t="str">
-        <f>V!A169</f>
-        <v/>
-      </c>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A90" t="str">
-        <f>V!A170</f>
-        <v/>
-      </c>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A91" t="str">
-        <f>V!A171</f>
-        <v/>
-      </c>
-    </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A92" t="str">
-        <f>V!A172</f>
-        <v/>
-      </c>
-    </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A93" t="str">
-        <f>V!A173</f>
-        <v/>
-      </c>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A94" t="str">
-        <f>V!A174</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Empties blank rows from input file
</commit_message>
<xml_diff>
--- a/InputData/plcy-schd/V/Vintage.xlsx
+++ b/InputData/plcy-schd/V/Vintage.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\plcy-schd\V\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A7A55AB-7E12-459F-B36D-DB5D5E1386B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD12AEC6-80C9-4241-9904-9376C77E7216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29580" yWindow="780" windowWidth="21600" windowHeight="11175" activeTab="1" xr2:uid="{70679913-52CE-4866-92D3-04053F7F27F8}"/>
+    <workbookView xWindow="29925" yWindow="1125" windowWidth="21600" windowHeight="11175" activeTab="5" xr2:uid="{70679913-52CE-4866-92D3-04053F7F27F8}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>

</xml_diff>